<commit_message>
Actualizar template ACT-122 segun instrucciones
</commit_message>
<xml_diff>
--- a/Documentos/ACT-122 CHO Instrucciones CELDAS EXCEL.xlsx
+++ b/Documentos/ACT-122 CHO Instrucciones CELDAS EXCEL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Enrique Saavedra\Documents\PROGRAMAS AI\Programa ACT\Documentos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\M2A (GD)\CARRETERAS\DOCUMENTOS CARRETERAS\FORMAS Y DOCUMENTOS ACT\Formas con celdas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CC894A-8152-4116-8A2E-8DCF9B3E9948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3008A4-1C46-4DF7-8A62-42EBC7360542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24" yWindow="252" windowWidth="18900" windowHeight="10896" xr2:uid="{CB186F85-06D1-4480-AABA-C5C6475F0F1E}"/>
+    <workbookView xWindow="-25320" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{CB186F85-06D1-4480-AABA-C5C6475F0F1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="78">
   <si>
     <t>Distribución de las copias de este documento</t>
   </si>
@@ -110,9 +110,6 @@
   </si>
   <si>
     <t>Número de la partida según indicado en el Desglose de Partidas incluido en el contrato (proposal).</t>
-  </si>
-  <si>
-    <t>Breve descripción del trabajo y/o las partidas incluidas en el documento incluyendo las estaciones donde se realizará el trabajo.</t>
   </si>
   <si>
     <t>Marcar todas las opciones que apliquen.</t>
@@ -520,6 +517,15 @@
   </si>
   <si>
     <t xml:space="preserve">J7 </t>
+  </si>
+  <si>
+    <t>Hoja 2</t>
+  </si>
+  <si>
+    <t>AZ60</t>
+  </si>
+  <si>
+    <t>Scope del trabajo y/o las partidas incluidas en el documento incluyendo las estaciones donde se realizará el trabajo.</t>
   </si>
 </sst>
 </file>
@@ -669,7 +675,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -692,6 +698,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -712,27 +733,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1073,7 +1073,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F54E80DF-BF7D-4BC9-802D-E3A0B42C2928}">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="12" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
@@ -1089,34 +1089,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="22.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="16"/>
+      <c r="A1" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="9"/>
     </row>
     <row r="2" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16" t="s">
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="16"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="9"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
@@ -1126,12 +1126,11 @@
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="J3" s="18"/>
+        <v>74</v>
+      </c>
     </row>
     <row r="4" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
@@ -1141,12 +1140,11 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J4" s="18"/>
+        <v>39</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
@@ -1156,12 +1154,11 @@
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J5" s="18"/>
+        <v>40</v>
+      </c>
     </row>
     <row r="6" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
@@ -1171,12 +1168,11 @@
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" s="18"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
@@ -1186,12 +1182,11 @@
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J7" s="18"/>
+        <v>42</v>
+      </c>
     </row>
     <row r="8" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
@@ -1201,52 +1196,47 @@
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="16">
+        <v>7</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="J8" s="18"/>
-    </row>
-    <row r="9" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="11">
-        <v>7</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>45</v>
-      </c>
       <c r="E9" s="7"/>
-      <c r="J9" s="18"/>
     </row>
     <row r="10" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="14"/>
+      <c r="A10" s="16"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="19"/>
       <c r="E10" s="7"/>
-      <c r="J10" s="18"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="14"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="19"/>
       <c r="E11" s="7"/>
-      <c r="J11" s="18"/>
     </row>
     <row r="12" spans="1:10" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="14"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="19"/>
       <c r="E12" s="7"/>
-      <c r="J12" s="18"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
@@ -1256,12 +1246,11 @@
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J13" s="18"/>
+        <v>47</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
@@ -1271,12 +1260,11 @@
         <v>1</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="J14" s="18"/>
+        <v>48</v>
+      </c>
     </row>
     <row r="15" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
@@ -1286,12 +1274,11 @@
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J15" s="18"/>
+        <v>49</v>
+      </c>
     </row>
     <row r="16" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
@@ -1301,27 +1288,25 @@
         <v>1</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="J16" s="18"/>
+        <v>50</v>
+      </c>
     </row>
     <row r="17" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="J17" s="18"/>
+        <v>51</v>
+      </c>
     </row>
     <row r="18" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
@@ -1331,12 +1316,11 @@
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="J18" s="18"/>
+        <v>52</v>
+      </c>
     </row>
     <row r="19" spans="1:10" ht="50.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
@@ -1346,12 +1330,12 @@
         <v>1</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="J19" s="19"/>
+        <v>52</v>
+      </c>
+      <c r="J19" s="7"/>
     </row>
     <row r="20" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
@@ -1361,12 +1345,12 @@
         <v>1</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="J20" s="19"/>
+        <v>53</v>
+      </c>
+      <c r="J20" s="7"/>
     </row>
     <row r="21" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
@@ -1376,12 +1360,12 @@
         <v>1</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="J21" s="19"/>
+        <v>54</v>
+      </c>
+      <c r="J21" s="7"/>
     </row>
     <row r="22" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
@@ -1391,12 +1375,12 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="J22" s="19"/>
+        <v>55</v>
+      </c>
+      <c r="J22" s="7"/>
     </row>
     <row r="23" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
@@ -1409,9 +1393,9 @@
         <v>4</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J23" s="19"/>
+        <v>61</v>
+      </c>
+      <c r="J23" s="7"/>
     </row>
     <row r="24" spans="1:10" ht="74.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
@@ -1423,7 +1407,6 @@
       <c r="C24" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J24" s="18"/>
     </row>
     <row r="25" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
@@ -1432,14 +1415,13 @@
       <c r="B25" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C25" s="18" t="s">
-        <v>37</v>
+      <c r="C25" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E25" s="4"/>
-      <c r="J25" s="18"/>
     </row>
     <row r="26" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
@@ -1448,8 +1430,8 @@
       <c r="B26" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>35</v>
+      <c r="C26" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
@@ -1459,11 +1441,11 @@
       <c r="B27" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C27" s="18" t="s">
-        <v>33</v>
+      <c r="C27" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
@@ -1473,11 +1455,11 @@
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C28" s="18" t="s">
-        <v>31</v>
+      <c r="C28" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
@@ -1487,11 +1469,11 @@
       <c r="B29" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="18" t="s">
-        <v>29</v>
+      <c r="C29" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
@@ -1501,11 +1483,11 @@
       <c r="B30" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
@@ -1515,25 +1497,25 @@
       <c r="B31" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="18" t="s">
-        <v>26</v>
+      <c r="C31" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>26</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C32" s="18" t="s">
-        <v>25</v>
+      <c r="C32" s="1" t="s">
+        <v>24</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1543,11 +1525,11 @@
       <c r="B33" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C33" s="18" t="s">
-        <v>24</v>
+      <c r="C33" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1557,11 +1539,11 @@
       <c r="B34" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C34" s="18" t="s">
-        <v>23</v>
+      <c r="C34" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
@@ -1571,11 +1553,11 @@
       <c r="B35" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C35" s="18" t="s">
-        <v>21</v>
+      <c r="C35" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
@@ -1585,11 +1567,11 @@
       <c r="B36" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C36" s="18" t="s">
-        <v>19</v>
+      <c r="C36" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
@@ -1599,11 +1581,11 @@
       <c r="B37" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C37" s="18" t="s">
-        <v>17</v>
+      <c r="C37" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57" x14ac:dyDescent="0.3">
@@ -1613,11 +1595,11 @@
       <c r="B38" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C38" s="18" t="s">
-        <v>15</v>
+      <c r="C38" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1627,11 +1609,11 @@
       <c r="B39" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C39" s="18" t="s">
-        <v>12</v>
+      <c r="C39" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1641,11 +1623,11 @@
       <c r="B40" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C40" s="18" t="s">
-        <v>10</v>
+      <c r="C40" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
@@ -1655,21 +1637,21 @@
       <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C41" s="20" t="s">
-        <v>8</v>
+      <c r="C41" s="18" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C42" s="20"/>
+      <c r="C42" s="18"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C43" s="20"/>
+      <c r="C43" s="18"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C44" s="20"/>
+      <c r="C44" s="18"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C45" s="20"/>
+      <c r="C45" s="18"/>
     </row>
     <row r="46" spans="1:4" ht="79.8" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
@@ -1678,11 +1660,11 @@
       <c r="B46" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C46" s="18" t="s">
+      <c r="C46" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="12.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1692,8 +1674,22 @@
       <c r="B47" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C47" s="21" t="s">
+      <c r="C47" s="11" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C50" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D50" s="1" t="str">
+        <f>_xlfn.CONCAT(J13, , J14)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completar integracion de celdas restantes en template ACT-122
</commit_message>
<xml_diff>
--- a/Documentos/ACT-122 CHO Instrucciones CELDAS EXCEL.xlsx
+++ b/Documentos/ACT-122 CHO Instrucciones CELDAS EXCEL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\M2A (GD)\CARRETERAS\DOCUMENTOS CARRETERAS\FORMAS Y DOCUMENTOS ACT\Formas con celdas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3008A4-1C46-4DF7-8A62-42EBC7360542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0FE7E40-8171-4FA8-87C2-779E1896CC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{CB186F85-06D1-4480-AABA-C5C6475F0F1E}"/>
+    <workbookView xWindow="-12705" yWindow="0" windowWidth="12810" windowHeight="15135" xr2:uid="{CB186F85-06D1-4480-AABA-C5C6475F0F1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="79">
   <si>
     <t>Distribución de las copias de este documento</t>
   </si>
@@ -459,9 +459,6 @@
     <t>B18 Y/O V18 Y/O AN18</t>
   </si>
   <si>
-    <t>B21:B26</t>
-  </si>
-  <si>
     <t>M44</t>
   </si>
   <si>
@@ -477,30 +474,9 @@
     <t>C68:BI107</t>
   </si>
   <si>
-    <t>B32:B36</t>
-  </si>
-  <si>
-    <t>H32:H36</t>
-  </si>
-  <si>
-    <t>AJ32:AJ36</t>
-  </si>
-  <si>
-    <t>AN32:AN36</t>
-  </si>
-  <si>
-    <t>AT32:AT36</t>
-  </si>
-  <si>
     <t>Monto total de la partida. Multiplicación de columna quantity y unit price</t>
   </si>
   <si>
-    <t>AZ32:AZ36</t>
-  </si>
-  <si>
-    <t>BF32:BF36</t>
-  </si>
-  <si>
     <t>AZ37</t>
   </si>
   <si>
@@ -526,6 +502,33 @@
   </si>
   <si>
     <t>Scope del trabajo y/o las partidas incluidas en el documento incluyendo las estaciones donde se realizará el trabajo.</t>
+  </si>
+  <si>
+    <t>B32:B36 y/o B39:b41</t>
+  </si>
+  <si>
+    <t>E32:e36 y/o E39:e41</t>
+  </si>
+  <si>
+    <t>H32:H36 y/o H39:h41</t>
+  </si>
+  <si>
+    <t>AJ32:AJ36 y/o aj39:aj41</t>
+  </si>
+  <si>
+    <t>AN32:AN36 y/o an39:an41</t>
+  </si>
+  <si>
+    <t>AT32:AT36 y/o at39:at41</t>
+  </si>
+  <si>
+    <t>AZ32:AZ36 y/o az39:az41</t>
+  </si>
+  <si>
+    <t>BF32:BF36 y/o bf39:bf41</t>
+  </si>
+  <si>
+    <t>B21</t>
   </si>
 </sst>
 </file>
@@ -1129,7 +1132,7 @@
         <v>37</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
@@ -1375,10 +1378,10 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="J22" s="7"/>
     </row>
@@ -1393,7 +1396,7 @@
         <v>4</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="J23" s="7"/>
     </row>
@@ -1407,8 +1410,11 @@
       <c r="C24" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D24" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>19</v>
       </c>
@@ -1419,7 +1425,7 @@
         <v>36</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="E25" s="4"/>
     </row>
@@ -1434,7 +1440,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>21</v>
       </c>
@@ -1445,10 +1451,10 @@
         <v>32</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>22</v>
       </c>
@@ -1459,10 +1465,10 @@
         <v>30</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>23</v>
       </c>
@@ -1473,10 +1479,10 @@
         <v>28</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>24</v>
       </c>
@@ -1484,13 +1490,13 @@
         <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>25</v>
       </c>
@@ -1501,7 +1507,7 @@
         <v>25</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1515,7 +1521,7 @@
         <v>24</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1529,7 +1535,7 @@
         <v>23</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1543,7 +1549,7 @@
         <v>22</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
@@ -1557,7 +1563,7 @@
         <v>20</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
@@ -1571,7 +1577,7 @@
         <v>18</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
@@ -1585,7 +1591,7 @@
         <v>16</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57" x14ac:dyDescent="0.3">
@@ -1599,7 +1605,7 @@
         <v>14</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1613,7 +1619,7 @@
         <v>11</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -1627,7 +1633,7 @@
         <v>9</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
@@ -1664,7 +1670,7 @@
         <v>2</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="12.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1680,12 +1686,12 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="12" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C50" s="1" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D50" s="1" t="str">
         <f>_xlfn.CONCAT(J13, , J14)</f>

</xml_diff>

<commit_message>
Correcciones de Reporte de CM y Actualización de ACT-122B (Rev 12-2024)
</commit_message>
<xml_diff>
--- a/Documentos/ACT-122 CHO Instrucciones CELDAS EXCEL.xlsx
+++ b/Documentos/ACT-122 CHO Instrucciones CELDAS EXCEL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\M2A (GD)\CARRETERAS\DOCUMENTOS CARRETERAS\FORMAS Y DOCUMENTOS ACT\Formas con celdas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0FE7E40-8171-4FA8-87C2-779E1896CC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7146F7-4861-48F3-8532-BD129D53CFB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-12705" yWindow="0" windowWidth="12810" windowHeight="15135" xr2:uid="{CB186F85-06D1-4480-AABA-C5C6475F0F1E}"/>
+    <workbookView xWindow="-14505" yWindow="-1830" windowWidth="14610" windowHeight="15585" xr2:uid="{CB186F85-06D1-4480-AABA-C5C6475F0F1E}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="90">
   <si>
     <t>Distribución de las copias de este documento</t>
   </si>
@@ -230,9 +230,6 @@
   </si>
   <si>
     <t>Nueva fecha de terminación (fecha proyectada incluyendo el tiempo en este documento y todas las extensiones de tiempo previamente aprobadas).</t>
-  </si>
-  <si>
-    <t>Nombre y firma del Supervisor de Proyecto/Gerente de Proyecto, Director de Distrito/Gerente de Programa y Director de la Oficina de Construcción.</t>
   </si>
   <si>
     <t xml:space="preserve"> De los días de extensión de tiempo otorgados en el encasillado 11, indique cuántos de ellos son compensables, de no haber días compensables indique N/A.</t>
@@ -432,9 +429,6 @@
     <t>TITULO</t>
   </si>
   <si>
-    <t>CELDA</t>
-  </si>
-  <si>
     <t>J14</t>
   </si>
   <si>
@@ -453,82 +447,121 @@
     <t>automatica</t>
   </si>
   <si>
-    <t>BA13</t>
-  </si>
-  <si>
-    <t>B18 Y/O V18 Y/O AN18</t>
-  </si>
-  <si>
-    <t>M44</t>
-  </si>
-  <si>
-    <t>M46</t>
-  </si>
-  <si>
     <t>M48</t>
   </si>
   <si>
     <t>M52</t>
   </si>
   <si>
-    <t>C68:BI107</t>
-  </si>
-  <si>
     <t>Monto total de la partida. Multiplicación de columna quantity y unit price</t>
   </si>
   <si>
-    <t>AZ37</t>
-  </si>
-  <si>
-    <t>AZ42</t>
-  </si>
-  <si>
-    <t>BA44</t>
-  </si>
-  <si>
-    <t>BA45</t>
-  </si>
-  <si>
-    <t>BA46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J7 </t>
-  </si>
-  <si>
     <t>Hoja 2</t>
   </si>
   <si>
-    <t>AZ60</t>
-  </si>
-  <si>
     <t>Scope del trabajo y/o las partidas incluidas en el documento incluyendo las estaciones donde se realizará el trabajo.</t>
   </si>
   <si>
-    <t>B32:B36 y/o B39:b41</t>
-  </si>
-  <si>
-    <t>E32:e36 y/o E39:e41</t>
-  </si>
-  <si>
-    <t>H32:H36 y/o H39:h41</t>
-  </si>
-  <si>
-    <t>AJ32:AJ36 y/o aj39:aj41</t>
-  </si>
-  <si>
-    <t>AN32:AN36 y/o an39:an41</t>
-  </si>
-  <si>
-    <t>AT32:AT36 y/o at39:at41</t>
-  </si>
-  <si>
-    <t>AZ32:AZ36 y/o az39:az41</t>
-  </si>
-  <si>
-    <t>BF32:BF36 y/o bf39:bf41</t>
-  </si>
-  <si>
-    <t>B21</t>
+    <t>J15</t>
+  </si>
+  <si>
+    <t>9a</t>
+  </si>
+  <si>
+    <t>Fecha del documento</t>
+  </si>
+  <si>
+    <t>ba11</t>
+  </si>
+  <si>
+    <t>ba14</t>
+  </si>
+  <si>
+    <t>B19 Y/O V19 Y/O AN19</t>
+  </si>
+  <si>
+    <t>B22</t>
+  </si>
+  <si>
+    <t>B35:B39 y/o B42:b44</t>
+  </si>
+  <si>
+    <t>E35:e39 y/o E42:e44</t>
+  </si>
+  <si>
+    <t>H35:H39 y/o H42:h44</t>
+  </si>
+  <si>
+    <t>AJ35:AJ39 y/o aj42:aj44</t>
+  </si>
+  <si>
+    <t>AN35:AN39 y/o an42:an44</t>
+  </si>
+  <si>
+    <t>AT35:AT39 y/o at42:at44</t>
+  </si>
+  <si>
+    <t>AZ35:AZ39 y/o az42:az44</t>
+  </si>
+  <si>
+    <t>BF35:BF39 y/o bf42:bf44</t>
+  </si>
+  <si>
+    <t>AZ40</t>
+  </si>
+  <si>
+    <t>AZ46</t>
+  </si>
+  <si>
+    <t>BA48</t>
+  </si>
+  <si>
+    <t>BA49</t>
+  </si>
+  <si>
+    <t>BA50</t>
+  </si>
+  <si>
+    <t>M50</t>
+  </si>
+  <si>
+    <t>M54</t>
+  </si>
+  <si>
+    <t>Director de Distrito/Gerente de Programa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Director de la Oficina de Construcción.</t>
+  </si>
+  <si>
+    <t>Nombre y firma del Supervisor de Proyecto/Gerente de Proyecto</t>
+  </si>
+  <si>
+    <t>AL52</t>
+  </si>
+  <si>
+    <t>M56</t>
+  </si>
+  <si>
+    <t>c72</t>
+  </si>
+  <si>
+    <t>AZ64</t>
+  </si>
+  <si>
+    <t>Hoja 1</t>
+  </si>
+  <si>
+    <t>k63</t>
+  </si>
+  <si>
+    <t>k64</t>
+  </si>
+  <si>
+    <t>az64</t>
+  </si>
+  <si>
+    <t>bc64</t>
   </si>
 </sst>
 </file>
@@ -1076,7 +1109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F54E80DF-BF7D-4BC9-802D-E3A0B42C2928}">
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="12" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
@@ -1093,7 +1126,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="22.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -1109,12 +1142,14 @@
       <c r="A2" s="8"/>
       <c r="B2" s="9"/>
       <c r="C2" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E2" s="9"/>
+        <v>85</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="F2" s="9"/>
       <c r="G2" s="9"/>
       <c r="H2" s="9"/>
@@ -1129,10 +1164,13 @@
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>66</v>
+        <v>38</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
@@ -1143,7 +1181,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>39</v>
@@ -1157,10 +1195,13 @@
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>40</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
@@ -1171,7 +1212,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>41</v>
@@ -1185,7 +1226,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>42</v>
@@ -1199,7 +1240,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>43</v>
@@ -1213,12 +1254,14 @@
         <v>1</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="7"/>
+        <v>45</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="10" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="16"/>
@@ -1249,270 +1292,273 @@
         <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A15" s="5">
+        <v>9</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A14" s="5">
-        <v>9</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C14" s="1" t="s">
+    <row r="16" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="5">
+        <v>10</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="5">
+        <v>11</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A19" s="5">
+        <v>12</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="50.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5">
+        <v>13</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J20" s="7"/>
+    </row>
+    <row r="21" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="5">
+        <v>14</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="J21" s="7"/>
+    </row>
+    <row r="22" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A22" s="5">
+        <v>15</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J22" s="7"/>
+    </row>
+    <row r="23" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="5">
+        <v>16</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J23" s="7"/>
+    </row>
+    <row r="24" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="5">
+        <v>17</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J24" s="7"/>
+    </row>
+    <row r="25" spans="1:10" ht="74.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="5">
+        <v>18</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1">
         <v>19</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="5">
-        <v>10</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="5">
-        <v>11</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A18" s="5">
-        <v>12</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="50.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5">
-        <v>13</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="J19" s="7"/>
-    </row>
-    <row r="20" spans="1:10" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="5">
-        <v>14</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="J20" s="7"/>
-    </row>
-    <row r="21" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A21" s="5">
-        <v>15</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="J21" s="7"/>
-    </row>
-    <row r="22" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5">
-        <v>16</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="J22" s="7"/>
-    </row>
-    <row r="23" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5">
-        <v>17</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J23" s="7"/>
-    </row>
-    <row r="24" spans="1:10" ht="74.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="5">
-        <v>18</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="34.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="1">
-        <v>19</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E25" s="4"/>
-    </row>
-    <row r="26" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A26" s="1">
+      <c r="B26" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
         <v>20</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1">
-        <v>21</v>
-      </c>
       <c r="B27" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
+        <v>24</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
         <v>25</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A32" s="1">
-        <v>26</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>1</v>
@@ -1521,12 +1567,12 @@
         <v>24</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>1</v>
@@ -1535,12 +1581,12 @@
         <v>23</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>1</v>
@@ -1549,151 +1595,181 @@
         <v>22</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
+        <v>30</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
         <v>31</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="57" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
+      <c r="B38" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="57" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
         <v>32</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
+      <c r="B39" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
         <v>33</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A40" s="1">
+      <c r="B40" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C41" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C42" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="34.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
         <v>34</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C40" s="1" t="s">
+      <c r="B43" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="1">
+      <c r="D43" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="1">
         <v>35</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C41" s="18" t="s">
+      <c r="B44" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C44" s="18" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C42" s="18"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C43" s="18"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C44" s="18"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C45" s="18"/>
     </row>
-    <row r="46" spans="1:4" ht="79.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="1">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C46" s="18"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C47" s="18"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C48" s="18"/>
+    </row>
+    <row r="49" spans="1:4" ht="79.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
         <v>36</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C46" s="1" t="s">
+      <c r="B49" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="12.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="4">
+      <c r="D49" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="12.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="4">
         <v>37</v>
       </c>
-      <c r="B47" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C47" s="11" t="s">
+      <c r="B50" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="11" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="12" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C50" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D50" s="1" t="str">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C53" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D53" s="1" t="str">
         <f>_xlfn.CONCAT(J13, , J14)</f>
         <v/>
       </c>
@@ -1704,7 +1780,7 @@
     <mergeCell ref="A9:A12"/>
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="C9:C12"/>
-    <mergeCell ref="C41:C45"/>
+    <mergeCell ref="C44:C48"/>
     <mergeCell ref="D9:D12"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>